<commit_message>
Update data layers Update suitability factor (and complete them) Added additional scenario for policy groups.
</commit_message>
<xml_diff>
--- a/lus_demo/data/Scenarioclaims/LUS_demo_additionalclaims.xlsx
+++ b/lus_demo/data/Scenarioclaims/LUS_demo_additionalclaims.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GeoDMS\ProjDir\LandUseModelling\lus_demo\data\Scenarioclaims\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ProjDir\_Archief\LandUseModelling\lus_demo\data\Scenarioclaims\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC9D8F5-934A-4F20-B6C9-B7ABFC3B2BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32F5F229-9EE1-4407-BFFD-0667F09048B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" activeTab="5" xr2:uid="{CBDA8ACD-4757-4B5C-80C6-60E6B82D6B8E}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" activeTab="5" xr2:uid="{CBDA8ACD-4757-4B5C-80C6-60E6B82D6B8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Residential" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="83">
   <si>
     <t>RstIntPer</t>
   </si>
@@ -290,6 +290,9 @@
   </si>
   <si>
     <t>Check sum</t>
+  </si>
+  <si>
+    <t>A1_Policy</t>
   </si>
 </sst>
 </file>
@@ -1306,13 +1309,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FAFA4DE-4904-4234-9879-BEB8EEB0E256}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1323,16 +1326,19 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1344,19 +1350,23 @@
         <v>0</v>
       </c>
       <c r="D2">
+        <f>C2</f>
+        <v>0</v>
+      </c>
+      <c r="E2">
         <f>Claims!D17</f>
         <v>0</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <f>Claims!E17</f>
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>Claims!F17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1368,19 +1378,23 @@
         <v>35178.417894101935</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:D5" si="0">C3</f>
+        <v>35178.417894101935</v>
+      </c>
+      <c r="E3">
         <f>Claims!D18</f>
         <v>22623.438363510089</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <f>Claims!E18</f>
         <v>16042.250229911986</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f>Claims!F18</f>
         <v>5197.8528249684841</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1392,19 +1406,23 @@
         <v>22640.084259384239</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
+        <v>22640.084259384239</v>
+      </c>
+      <c r="E4">
         <f>Claims!D19</f>
         <v>14657.985714878037</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f>Claims!E19</f>
         <v>8658.8220384302585</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f>Claims!F19</f>
         <v>4876.8138416981838</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1416,14 +1434,18 @@
         <v>14270.497846513825</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
+        <v>14270.497846513825</v>
+      </c>
+      <c r="E5">
         <f>Claims!D20</f>
         <v>9342.5759216118695</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f>Claims!E20</f>
         <v>5522.9277316577554</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f>Claims!F20</f>
         <v>0</v>
       </c>
@@ -1435,13 +1457,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4028A29-9BA4-469D-8E81-4AC11527BD57}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1452,16 +1474,19 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1473,19 +1498,23 @@
         <v>0</v>
       </c>
       <c r="D2">
+        <f>C2</f>
+        <v>0</v>
+      </c>
+      <c r="E2">
         <f>Claims!H17</f>
         <v>0</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <f>Claims!I17</f>
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>Claims!J17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1497,19 +1526,23 @@
         <v>8564.6583762471237</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:D5" si="0">C3</f>
+        <v>8564.6583762471237</v>
+      </c>
+      <c r="E3">
         <f>Claims!H18</f>
         <v>3194.2349491638129</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <f>Claims!I18</f>
         <v>2858.9768934498156</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f>Claims!J18</f>
         <v>2858.9768928864987</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1521,19 +1554,23 @@
         <v>7786.8225183947834</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
+        <v>7786.8225183947834</v>
+      </c>
+      <c r="E4">
         <f>Claims!H19</f>
         <v>5803.5854614490017</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f>Claims!I19</f>
         <v>2018.8675099725217</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f>Claims!J19</f>
         <v>2018.86751025475</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1545,14 +1582,18 @@
         <v>7869.769105358092</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
+        <v>7869.769105358092</v>
+      </c>
+      <c r="E5">
         <f>Claims!H20</f>
         <v>6818.429589387184</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f>Claims!I20</f>
         <v>2534.6555965776624</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f>Claims!J20</f>
         <v>2534.6555968587509</v>
       </c>
@@ -1564,13 +1605,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA1C4D6-D08C-4574-80C3-050D11BF327D}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1581,16 +1622,19 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1602,19 +1646,23 @@
         <v>0</v>
       </c>
       <c r="D2">
+        <f>C2</f>
+        <v>0</v>
+      </c>
+      <c r="E2">
         <f>Claims!L17</f>
         <v>0</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <f>Claims!M17</f>
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>Claims!N17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1626,19 +1674,23 @@
         <v>16276.728473224881</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:D5" si="0">C3</f>
+        <v>16276.728473224881</v>
+      </c>
+      <c r="E3">
         <f>Claims!L18</f>
         <v>13458.317044969379</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <f>Claims!M18</f>
         <v>8361.5338065092637</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f>Claims!N18</f>
         <v>3339.3601603774682</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1650,19 +1702,23 @@
         <v>8679.5726379710923</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
+        <v>8679.5726379710923</v>
+      </c>
+      <c r="E4">
         <f>Claims!L19</f>
         <v>4856.6829550306202</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f>Claims!M19</f>
         <v>2916.1861705639703</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f>Claims!N19</f>
         <v>576.63983962253212</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1674,14 +1730,18 @@
         <v>3556.698888804031</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
+        <v>3556.698888804031</v>
+      </c>
+      <c r="E5">
         <f>Claims!L20</f>
         <v>0</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f>Claims!M20</f>
         <v>470.28002292676678</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f>Claims!N20</f>
         <v>0</v>
       </c>
@@ -1693,13 +1753,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A478943-3230-4275-A5A2-91A3DE9E7B8A}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1710,16 +1770,19 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1731,19 +1794,23 @@
         <v>0</v>
       </c>
       <c r="D2">
+        <f>C2</f>
+        <v>0</v>
+      </c>
+      <c r="E2">
         <f>Claims!P17</f>
         <v>0</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <f>Claims!Q17</f>
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>Claims!R17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1755,19 +1822,23 @@
         <v>7934.5605090314539</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:D5" si="0">C3</f>
+        <v>7934.5605090314539</v>
+      </c>
+      <c r="E3">
         <f>Claims!P18</f>
         <v>7789.4979175677599</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <f>Claims!Q18</f>
         <v>15736.945790174215</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f>Claims!R18</f>
         <v>12524.908345319693</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1779,19 +1850,23 @@
         <v>14107.958280723678</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
+        <v>14107.958280723678</v>
+      </c>
+      <c r="E4">
         <f>Claims!P19</f>
         <v>15061.112157672052</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f>Claims!Q19</f>
         <v>30439.557722305552</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f>Claims!R19</f>
         <v>31578.457555692534</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1803,14 +1878,18 @@
         <v>12957.481210244869</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
+        <v>12957.481210244869</v>
+      </c>
+      <c r="E5">
         <f>Claims!P20</f>
         <v>12149.389924760186</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f>Claims!Q20</f>
         <v>24823.496487520242</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f>Claims!R20</f>
         <v>26896.634098987779</v>
       </c>
@@ -1822,13 +1901,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B564767-4407-4477-931B-2AF14AA45329}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1839,16 +1918,19 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1860,19 +1942,23 @@
         <v>0</v>
       </c>
       <c r="D2">
+        <f>C2</f>
+        <v>0</v>
+      </c>
+      <c r="E2">
         <f>Claims!X17</f>
         <v>0</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <f>Claims!Y17</f>
         <v>0</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>Claims!Z17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1884,19 +1970,23 @@
         <v>-53530.001361996634</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:D5" si="0">C3</f>
+        <v>-53530.001361996634</v>
+      </c>
+      <c r="E3">
         <f>Claims!X18</f>
         <v>-32871.257853391544</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <f>Claims!Y18</f>
         <v>-34900.459981103893</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f>Claims!Z18</f>
         <v>-16033.019536105601</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1908,19 +1998,23 @@
         <v>-49002.947188209138</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
+        <v>-49002.947188209138</v>
+      </c>
+      <c r="E4">
         <f>Claims!X19</f>
         <v>-37314.182053772573</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f>Claims!Y19</f>
         <v>-37377.308813142532</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f>Claims!Z19</f>
         <v>-30461.018438075833</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1932,14 +2026,18 @@
         <v>-35840.05144979422</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
+        <v>-35840.05144979422</v>
+      </c>
+      <c r="E5">
         <f>Claims!X20</f>
         <v>-24119.560092835884</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f>Claims!Y20</f>
         <v>-26656.231205753582</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f>Claims!Z20</f>
         <v>-24458.962025818568</v>
       </c>
@@ -1951,13 +2049,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE7080A5-74A6-455E-B147-F3205C83B262}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1968,16 +2066,19 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1989,19 +2090,23 @@
         <v>-15</v>
       </c>
       <c r="D2">
+        <f>C2</f>
+        <v>-15</v>
+      </c>
+      <c r="E2">
         <f>Claims!T17</f>
         <v>-15</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <f>Claims!U17</f>
         <v>-15</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>Claims!V17</f>
         <v>-15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2013,19 +2118,23 @@
         <v>-8287</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:D5" si="0">C3</f>
+        <v>-8287</v>
+      </c>
+      <c r="E3">
         <f>Claims!T18</f>
         <v>-8287</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <f>Claims!U18</f>
         <v>-8287</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f>Claims!V18</f>
         <v>-8287</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2037,19 +2146,23 @@
         <v>-6079</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
+        <v>-6079</v>
+      </c>
+      <c r="E4">
         <f>Claims!T19</f>
         <v>-6079</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f>Claims!U19</f>
         <v>-6079</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f>Claims!V19</f>
         <v>-6079</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2061,14 +2174,18 @@
         <v>-7069</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
+        <v>-7069</v>
+      </c>
+      <c r="E5">
         <f>Claims!T20</f>
         <v>-7069</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f>Claims!U20</f>
         <v>-7069</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f>Claims!V20</f>
         <v>-7069</v>
       </c>

</xml_diff>